<commit_message>
Preencher dashboard com formulário correto da Mobilize
</commit_message>
<xml_diff>
--- a/formulario/F.O.091.GOCO - Analise de Maturidade em Processos.xlsx
+++ b/formulario/F.O.091.GOCO - Analise de Maturidade em Processos.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,7 +501,7 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Padrão</t>
+          <t xml:space="preserve"> Padrão</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
@@ -511,25 +511,35 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Documentação</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Observação</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Plano de Ação</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Responsável</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Prazo</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Status da Ação</t>
         </is>
@@ -537,12 +547,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -551,12 +559,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>D.C.231.EXTE</t>
+          <t>D.C.231.EXTE - Emissão de boletos e duvidas frequêntes</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -569,47 +577,55 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
+          <t>Observação</t>
         </is>
       </c>
       <c r="L2" t="n">
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Divergências de versão e datas</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Corrigir D.C.231.EXTE</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>86.76470588235294</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Responsáveis documentais</t>
+          <t>NC 01: divergências de versão e data; o relatório não identifica a frente, o processo nem a data válida. Data da avaliação registrada pelo cabeçalho: 18/09/2026; o rodapé do relatório indica 16/09/2026.</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Validar versão, data e código do documento; atualizar o repositório e preservar a rastreabilidade.</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
+        <is>
+          <t>Equipe de processos</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>Aguardando ação</t>
         </is>
@@ -617,12 +633,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -631,12 +645,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>D.C.232.EXTE</t>
+          <t>D.C.232.EXTE - Reclamações de boletos</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -649,47 +663,55 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
+          <t>Observação</t>
         </is>
       </c>
       <c r="L3" t="n">
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Divergências de versão e datas</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Corrigir D.C.232.EXTE</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>86.76470588235294</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Responsáveis documentais</t>
+          <t>NC 01: divergências de versão e data; o relatório não identifica a frente, o processo nem a data válida.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Validar versão, data e código do documento; atualizar o repositório e preservar a rastreabilidade.</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
+        <is>
+          <t>Equipe de processos</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>Aguardando ação</t>
         </is>
@@ -697,12 +719,10 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -711,12 +731,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D.C.1504.EXTE</t>
+          <t>Documento de encerramento de leasing — sem código</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -729,47 +749,58 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
+          <t>Conformidade</t>
         </is>
       </c>
       <c r="L4" t="n">
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Datas duplicadas</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Corrigir D.C.1504.EXTE</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>86.76470588235294</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Responsáveis documentais</t>
+          <t>NC 02: documento existente sem código de identificação. Também não foi demonstrado critério formal para uso do processo manual.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Atribuir código, formalizar o critério de elegibilidade e exceção do processo manual, aprovar e publicar a versão vigente.</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
+        <is>
+          <t>Supervisão do Banco Mobilize</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
         <is>
           <t>Aguardando ação</t>
         </is>
@@ -777,12 +808,10 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -791,12 +820,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>D.C.2480.EXTE</t>
+          <t>Documento de rescisão de leasing — sem código</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -809,47 +838,58 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
+          <t>Conformidade</t>
         </is>
       </c>
       <c r="L5" t="n">
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Atualizado sem controle de versão</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Corrigir D.C.2480.EXTE</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>86.76470588235294</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Responsáveis documentais</t>
+          <t>NC 02: documento existente sem código de identificação. Também não foi demonstrado critério formal para uso do processo manual.</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Atribuir código, formalizar o critério de elegibilidade e exceção do processo manual, aprovar e publicar a versão vigente.</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
+        <is>
+          <t>Supervisão do Banco Mobilize</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>Aguardando ação</t>
         </is>
@@ -857,12 +897,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -871,12 +909,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>D.C.1517.EXTE</t>
+          <t>D.C.1504.EXTE - Promessa de pagamento e baixa de pagamento</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -889,47 +927,58 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
+          <t>Conformidade</t>
         </is>
       </c>
       <c r="L6" t="n">
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Controles de versão duplicados</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Corrigir D.C.1517.EXTE</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>86.76470588235294</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Responsáveis documentais</t>
+          <t>NC 03: datas de criação, modificação e aprovação duplicadas; o relatório não informa processo ou frente.</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Corrigir as datas e validar a trilha de criação, modificação e aprovação no controle documental.</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
+        <is>
+          <t>Equipe de processos</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>Aguardando ação</t>
         </is>
@@ -937,12 +986,10 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -951,12 +998,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>D.C.136.EXTE</t>
+          <t>D.C.2480.EXTE</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -969,47 +1016,58 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
+          <t>Conformidade</t>
         </is>
       </c>
       <c r="L7" t="n">
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Fluxograma descrito como orientação</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>Corrigir D.C.136.EXTE</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>86.76470588235294</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Responsáveis documentais</t>
+          <t>NC 04: documento atualizado sem alteração do controle de versão; a data da atualização não foi informada no relatório.</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Regularizar o controle de versão e registrar a data, aprovação e comunicação da versão vigente.</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
+        <is>
+          <t>Equipe de processos</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>Aguardando ação</t>
         </is>
@@ -1017,12 +1075,10 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1031,12 +1087,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Política</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Política da Informação Documentada</t>
+          <t>D.C.1517.EXTE - Pró-rata e mensalidade</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1052,11 +1108,6 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2025-01-25</t>
-        </is>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -1079,20 +1130,44 @@
       <c r="O8" t="n">
         <v>1</v>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Política da Informação Documentada - Documentação</t>
+      <c r="P8" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>NC 05: controles de versão duplicados; o relatório não informa processo, frente ou data válida.</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Eliminar a duplicidade, confirmar a versão vigente e atualizar o controle documental.</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Equipe de processos</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1101,12 +1176,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Procedimento</t>
+          <t>Backoffice Locadora — N2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Procedimento Operacional</t>
+          <t>D.C.136.EXTE - Seguros e Sinistros</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1122,11 +1197,6 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2025-01-25</t>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -1134,24 +1204,822 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>O documento é denominado fluxograma, mas foi descrito como material de orientação ou passo a passo. Processo, frente e atualização não foram informados.</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Validar a classificação documental, o conteúdo, a versão vigente e o vínculo com o processo aplicável.</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Equipe de processos</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Backoffice Locadora — N2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>P.O.498.OPER - Orientação quanto a solicitação de cancelamento</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>A orientação relativa aos dias adicionais após cinco dias na devolução do veículo não foi localizada.</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Elaborar ou localizar a orientação, aprovar, versionar e disponibilizar na Wiki vigente.</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Equipe de processos</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Backoffice — Banco N2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>D.C.016.EXTE - Kit pós aprovado - Cessão de direitos</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>A sequência documental deve ser explicitada e os SLAs por fila precisam ser confirmados.</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Organizar a cadeia documental por etapa, confirmar os SLAs e publicar a referência vigente.</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Jeferson Oliveira</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Backoffice — Banco N2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>D.C.017.EXTE - Imput da proposta Connect</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>Conformidade</t>
         </is>
       </c>
-      <c r="L9" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" t="n">
-        <v>1</v>
-      </c>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" t="n">
-        <v>1</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Procedimento Operacional - Documentação</t>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Organizar a cadeia documental por etapa, confirmar os SLAs e publicar a referência vigente.</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Jeferson Oliveira</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Backoffice — Locadora N2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>P.O.523.OPER - ORIENTAR QUANTO A SOLICITAÇÃO CONTESTAÇÃO - INFRAÇÃO TRÂNSITO</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Conformidade</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Organizar a cadeia documental por etapa, confirmar os SLAs e publicar a referência vigente.</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Jeferson Oliveira</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Backoffice — Locadora N2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>P.O.535.OPER - ORIENTAR QUANTO A SOLICITAÇÃO DE RECORRER A INFRAÇÃO</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Conformidade</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Organizar a cadeia documental por etapa, confirmar os SLAs e publicar a referência vigente.</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Jeferson Oliveira</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Backoffice — Locadora N2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>D.C.1337.EXTE -INFRAÇÕES DE TRÂNSITO</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Conformidade</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Organizar a cadeia documental por etapa, confirmar os SLAs e publicar a referência vigente.</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Jeferson Oliveira</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Clube FIQ</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>I.T.179.OPER - ORIENTAR QUANTO A TRATATIVA DE CLIENTES VIA CHAT</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Não Conformidade</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Wikis desatualizadas e ausência de classificação de criticidade consolidada para todos os processos.</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Atualizar Wikis e scripts, consolidar a criticidade e registrar aprovação, versão e vigência.</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Gestão do Clube FIQ e Processos</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Clube FIQ</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>I.T.176.OPER - ORIENTAR QUANTO A TRATATIVA DE INCENTIVO AO PORTAL</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Não Conformidade</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Wikis desatualizadas e ausência de classificação de criticidade consolidada para todos os processos.</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Atualizar Wikis e scripts, consolidar a criticidade e registrar aprovação, versão e vigência.</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Gestão do Clube FIQ e Processos</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>928734</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mobilize</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Clube FIQ</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>D.C.587.OPER - SCRIPT DE INCENTIVO AO PORTAL</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Não Conformidade</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>86.76470588235294</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Wikis desatualizadas e ausência de classificação de criticidade consolidada para todos os processos.</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Atualizar Wikis e scripts, consolidar a criticidade e registrar aprovação, versão e vigência.</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Gestão do Clube FIQ e Processos</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
         </is>
       </c>
     </row>
@@ -1290,7 +2158,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1351,7 +2219,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1415,7 +2283,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1479,7 +2347,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1543,7 +2411,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1607,7 +2475,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1671,7 +2539,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1735,7 +2603,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1799,7 +2667,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Backoffice</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1863,7 +2731,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1927,7 +2795,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1991,7 +2859,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2055,7 +2923,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2119,7 +2987,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2183,7 +3051,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2247,7 +3115,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2311,7 +3179,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2375,7 +3243,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>banco</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2875,7 +3743,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2939,7 +3807,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3003,7 +3871,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3067,7 +3935,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -3131,7 +3999,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3195,7 +4063,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3259,7 +4127,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3323,7 +4191,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3387,7 +4255,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Locadora</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3448,7 +4316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3504,58 +4372,86 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Conforme?</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Existência</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Padrão</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Conformidade</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Plano de Ação</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Responsável</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Prazo</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Status da Ação</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>Coerência</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Aplicação</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Atualização</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Conformidade</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Observação</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Plano de Ação</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Responsável</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Prazo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Status da Ação</t>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Score Treinamento</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -3564,12 +4460,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Treinamento</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Treinamento - Banco N1</t>
+          <t>Material de treinamento e reciclagem — Banco N1</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -3577,7 +4473,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -3585,57 +4481,72 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>NC 08: material existente sem controle de versão e sem evidência individual completa da reciclagem. Atualização e padronização não foram demonstradas.</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Versionar o material, vincular as fontes vigentes e completar a evidência individual da reciclagem.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Daniel da Silva</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="X2" t="n">
         <v>0</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Y2" t="n">
         <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Material sem controle de versão</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Versionar Treinamento - Banco N1</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Daniel da Silva</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Aguardando ação</t>
-        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3644,12 +4555,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Treinamento</t>
+          <t>Locadora — N1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Treinamento - Locadora N1</t>
+          <t>Material e plano de treinamento — Locadora N1</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -3665,57 +4576,72 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Não Conformidade</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>1</v>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
       </c>
       <c r="L3" t="n">
         <v>1</v>
       </c>
       <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>100</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Há planos e materiais, porém faltou rastreabilidade da evidência individual. Atualização e padronização não foram demonstradas de forma suficiente.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Vincular fontes vigentes, registrar versão e manter evidência individual da aplicação e reciclagem.</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Daniel da Silva</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
         <v>0</v>
       </c>
-      <c r="N3" t="n">
+      <c r="X3" t="n">
         <v>0</v>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Faltou rastreabilidade da evidência</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Versionar Treinamento - Locadora N1</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Daniel da Silva</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Aguardando ação</t>
-        </is>
+      <c r="Y3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3724,12 +4650,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Treinamento</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Treinamento - BackOffice N2</t>
+          <t>Estrutura de treinamento — BackOffice N2</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -3745,18 +4671,15 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Conformidade</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>1</v>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -3767,140 +4690,45 @@
       <c r="N4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Estrutura compatível</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Mobilize</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Treinamento</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Integração de Novos Colaboradores</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Conformidade</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Processo de integração</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Mobilize</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Treinamento</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Gestão de Incidentes</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Conformidade</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Treinamento de gestão de incidentes</t>
-        </is>
+      <c r="P4" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>100</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>A estrutura foi considerada compatível, mas o relatório não apresenta data de atualização nem evidência suficiente de padronização do material.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Manter a estrutura e complementar os registros de atualização, versão, padrão e fontes utilizadas.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Daniel da Silva</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3914,7 +4742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3965,33 +4793,86 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Conforme?</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Conforme?</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Existência</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Padrão</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Conformidade</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Plano de Ação</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Responsável</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Prazo</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Status da Ação</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
         <is>
           <t>Abrangência</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Conformidade</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Observação</t>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Score Qualidade</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -4000,12 +4881,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Qualidade</t>
+          <t>Banco — N1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Portal da Qualidade</t>
+          <t>Monitoria — Encerramento de leasing</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -4018,37 +4899,75 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Amostral</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Conformidade</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.5</v>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Não Conformidade</t>
+        </is>
       </c>
       <c r="L2" t="n">
         <v>1</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Monitoria Portal da Qualidade: Amostral</t>
-        </is>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>A monitoria existe, porém o formulário é genérico e não possui avaliação específica para Encerramento de Leasing. O processo é avaliado de modo geral, com foco em FCR, informações corretas e classificação para N2. A Wiki foi vista como base, mas não foi evidenciada sua utilização na contestação ou resposta à operação. O formulário 'Back Office Banco / Locadora - Checklist 2025' não possui histórico de atualização ou aprovação, nem rotina de revisão.</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Criar critérios específicos para Encerramento de Leasing; separar requisitos comportamentais e processuais; formalizar revisão, aprovação e histórico do checklist; exigir evidência da referência utilizada em contestação e resposta.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Qualidade e operação</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -4057,12 +4976,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Qualidade</t>
+          <t>Backoffice — N2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cessão de Direitos</t>
+          <t>Monitoria — Cessão de Direitos</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -4075,37 +4994,75 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Amostral</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Conformidade</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.5</v>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Não Conformidade</t>
+        </is>
       </c>
       <c r="L3" t="n">
         <v>1</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Monitoria Cessão de Direitos: Amostral</t>
-        </is>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>A monitoria existe e a avaliação registrada recebeu nota 100. Entretanto, o formulário é genérico para Banco e Locadora e não separa aspectos comportamentais e processuais solicitados pela operação. Foram evidenciados acompanhamento de telas e consulta à Wiki 'Cessão de Direitos - dúvidas e informações'. O documento D.C.198.EXTE, versão 2.0, de 21/06/2024, apresenta problema na data de edição.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Revisar e aprovar o checklist; criar critérios específicos por frente e processo; separar itens comportamentais e processuais; corrigir e validar a data de edição do D.C.198.EXTE; estabelecer rotina de atualização.</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Qualidade e operação</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
+        <v>928734</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -4114,12 +5071,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Qualidade</t>
+          <t>Clube FIQ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Clube FIQ</t>
+          <t>Monitoria — Clube FIQ</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -4130,29 +5087,50 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Não realizada</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Não Conformidade Grave</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
+      <c r="P4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Monitoria Clube FIQ: Não realizada</t>
-        </is>
+      <c r="Q4" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Não há monitoria do Clube FIQ há três meses devido à reformulação em andamento.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Retomar as monitorias após a definição dos novos fluxos; formalizar critérios, formulário, frequência, responsável e aprovação.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Qualidade e gestão do Clube FIQ</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Aguardando ação</t>
+        </is>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4209,7 +5187,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
@@ -4230,7 +5208,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
@@ -4251,7 +5229,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
@@ -4314,7 +5292,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
@@ -4335,7 +5313,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">

</xml_diff>

<commit_message>
Corrigir score Qualidade - mapear colunas corretas no data_loader
</commit_message>
<xml_diff>
--- a/formulario/F.O.091.GOCO - Analise de Maturidade em Processos.xlsx
+++ b/formulario/F.O.091.GOCO - Analise de Maturidade em Processos.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -4742,7 +4743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4778,29 +4779,29 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Foram feitas monitorias de qualidade?</t>
+          <t>Existe?</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Como são feitas as monitorias?</t>
+          <t>Está atualizado?</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Última atualização</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Padronizado?</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Conforme?</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Conforme?</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Conforme?</t>
-        </is>
-      </c>
       <c r="L1" t="inlineStr">
         <is>
           <t>Existência</t>
@@ -4854,16 +4855,6 @@
       <c r="V1" t="inlineStr">
         <is>
           <t>Status da Ação</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Abrangência</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Score Qualidade</t>
         </is>
       </c>
     </row>
@@ -4902,6 +4893,7 @@
           <t>SIM</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -4955,12 +4947,6 @@
           <t>Aguardando ação</t>
         </is>
       </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -4997,6 +4983,7 @@
           <t>SIM</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -5050,12 +5037,6 @@
           <t>Aguardando ação</t>
         </is>
       </c>
-      <c r="W3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -5087,6 +5068,9 @@
           <t>NÃO</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Observação</t>
@@ -5095,6 +5079,11 @@
       <c r="L4" t="n">
         <v>0</v>
       </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>0.5</v>
+      </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
@@ -5125,12 +5114,6 @@
         <is>
           <t>Aguardando ação</t>
         </is>
-      </c>
-      <c r="W4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5154,9 +5137,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -5168,7 +5148,6 @@
           <t>Resultado</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Faixa do Score</t>
@@ -5189,7 +5168,6 @@
       <c r="B4" t="n">
         <v>17</v>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>0-25</t>
@@ -5210,7 +5188,6 @@
       <c r="B5" t="n">
         <v>17</v>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>26-35</t>
@@ -5231,7 +5208,6 @@
       <c r="B6" t="n">
         <v>14</v>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>0-25</t>
@@ -5252,7 +5228,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>26-35</t>
@@ -5273,7 +5248,6 @@
       <c r="B8" t="n">
         <v>34</v>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>26-35</t>
@@ -5294,7 +5268,6 @@
       <c r="B9" t="n">
         <v>3</v>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>26-35</t>
@@ -5315,7 +5288,6 @@
       <c r="B10" t="n">
         <v>3</v>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>26-35</t>
@@ -5336,7 +5308,6 @@
       <c r="B11" t="n">
         <v>3</v>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>26-35</t>
@@ -5357,7 +5328,6 @@
       <c r="B12" t="n">
         <v>2</v>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>26-35</t>

</xml_diff>

<commit_message>
Corrigir Treinamento Conforme?.1, Indicadores mapear 'Conforme?' ao inves de 'Conformidade', Observacao=0.5, alinhar datas para 2026-09-18
</commit_message>
<xml_diff>
--- a/formulario/F.O.091.GOCO - Analise de Maturidade em Processos.xlsx
+++ b/formulario/F.O.091.GOCO - Analise de Maturidade em Processos.xlsx
@@ -2150,7 +2150,7 @@
         <v>928734</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2199,19 +2199,25 @@
       <c r="M2" t="n">
         <v>1</v>
       </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
         <v>100</v>
       </c>
       <c r="P2" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>928734</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2269,13 +2275,18 @@
       <c r="P3" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>928734</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2333,13 +2344,18 @@
       <c r="P4" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>928734</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -2397,13 +2413,18 @@
       <c r="P5" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>928734</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2461,13 +2482,18 @@
       <c r="P6" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>928734</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2525,13 +2551,18 @@
       <c r="P7" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
         <v>928734</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -2589,13 +2620,18 @@
       <c r="P8" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>928734</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -2653,13 +2689,18 @@
       <c r="P9" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>928734</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -2717,13 +2758,18 @@
       <c r="P10" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
         <v>928734</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -2781,13 +2827,18 @@
       <c r="P11" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
         <v>928734</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -2845,13 +2896,18 @@
       <c r="P12" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>928734</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -2909,13 +2965,18 @@
       <c r="P13" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>928734</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -2973,13 +3034,18 @@
       <c r="P14" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
         <v>928734</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -3037,13 +3103,18 @@
       <c r="P15" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
         <v>928734</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -3101,13 +3172,18 @@
       <c r="P16" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>928734</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -3165,13 +3241,18 @@
       <c r="P17" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
         <v>928734</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -3229,13 +3310,18 @@
       <c r="P18" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
         <v>928734</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -3293,13 +3379,18 @@
       <c r="P19" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
         <v>928734</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -3348,19 +3439,25 @@
       <c r="M20" t="n">
         <v>1</v>
       </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
         <v>100</v>
       </c>
       <c r="P20" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
         <v>928734</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -3409,19 +3506,25 @@
       <c r="M21" t="n">
         <v>1</v>
       </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
         <v>100</v>
       </c>
       <c r="P21" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
         <v>928734</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -3470,19 +3573,25 @@
       <c r="M22" t="n">
         <v>1</v>
       </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
         <v>100</v>
       </c>
       <c r="P22" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>928734</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -3531,19 +3640,25 @@
       <c r="M23" t="n">
         <v>1</v>
       </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
         <v>100</v>
       </c>
       <c r="P23" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>928734</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -3601,13 +3716,18 @@
       <c r="P24" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
         <v>928734</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -3665,13 +3785,18 @@
       <c r="P25" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>928734</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -3729,13 +3854,18 @@
       <c r="P26" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>928734</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -3793,13 +3923,18 @@
       <c r="P27" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
         <v>928734</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3857,13 +3992,18 @@
       <c r="P28" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>928734</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3921,13 +4061,18 @@
       <c r="P29" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
         <v>928734</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3985,13 +4130,18 @@
       <c r="P30" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
         <v>928734</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -4049,13 +4199,18 @@
       <c r="P31" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
         <v>928734</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -4113,13 +4268,18 @@
       <c r="P32" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
         <v>928734</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -4177,13 +4337,18 @@
       <c r="P33" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
         <v>928734</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -4241,13 +4406,18 @@
       <c r="P34" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
         <v>928734</v>
       </c>
       <c r="B35" s="2" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -4305,6 +4475,11 @@
       <c r="P35" t="n">
         <v>96.32352941176471</v>
       </c>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4893,7 +5068,6 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -4983,7 +5157,6 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -5068,9 +5241,6 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Observação</t>
@@ -5079,8 +5249,6 @@
       <c r="L4" t="n">
         <v>0</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
         <v>0.5</v>
       </c>

</xml_diff>